<commit_message>
feat: v6 model — log target, OOF encoding, interaction features (RMSE 22,124)
- Add 05_advanced_tuning.ipynb: log-transform target, per-fold OOF town encoding,
  three interaction features (dist_x_storey, lease_x_area, log_dist_to_cbd)
- Add sub_v6_log_blend.csv submission (Kaggle RMSE 22,124.05, CV 21,818)
- Update 04_model_tuning.ipynb: add LGBM tuning, blend search, v5 submission cells
- Add feature_engineering_explained and model_tuning_explained (md + html)
- Update submission tracker: add v6, remove duplicate v2 row
- Update README and CHANGELOG with v6 as new best

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/submission_tracker.xlsx
+++ b/outputs/submission_tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="SCORES" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="LEGEND" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SCORES" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEGEND" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -103,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -135,6 +135,8 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -664,182 +666,182 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>v2</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>2026-04-21</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>RF + Feature Engineering</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>03_feature_engineering.ipynb</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>Added: remaining_lease, dist_to_cbd, is_mature_estate, cyclical month, total_sold, rental_ratio, floor_area_per_room, town_median_price, amenity_score</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>n_estimators=100, max_depth=15, min_samples_leaf=5</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>26564</v>
-      </c>
-      <c r="H4" s="6" t="n">
-        <v>27582.06</v>
-      </c>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>Score worse than v1. RF already captured lat/lon and age implicitly.</t>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>XGBoost Tuned + Feature Eng</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>04_model_tuning.ipynb</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Same 11 engineered features. Switched from RF to XGBoost with RandomizedSearchCV tuning.</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>n_estimators=1000, max_depth=7, lr=0.05, subsample=0.7, colsample_bytree=0.6, min_child_weight=3</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>22748</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>22800.92</v>
+      </c>
+      <c r="I4" s="7" t="n"/>
+      <c r="J4" s="7" t="n"/>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>Best score so far. -3,142 vs v1 baseline. Gradient boosting + feature engineering working well together.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>v3</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>2026-04-21</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>XGBoost Tuned + Feature Eng</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>LightGBM Default + Feature Eng</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>04_model_tuning.ipynb</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>Same 11 engineered features. Switched from RF to XGBoost with RandomizedSearchCV tuning.</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>n_estimators=1000, max_depth=7, lr=0.05, subsample=0.7, colsample_bytree=0.6, min_child_weight=3</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="n">
-        <v>22748</v>
-      </c>
-      <c r="H5" s="4" t="n">
-        <v>22800.92</v>
-      </c>
-      <c r="I5" s="7" t="n"/>
-      <c r="J5" s="7" t="n"/>
-      <c r="K5" s="7" t="inlineStr">
-        <is>
-          <t>Best score so far. -3,142 vs v1 baseline. Gradient boosting + feature engineering working well together.</t>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Same 11 engineered features as v3. LightGBM with default params (no tuning).</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>n_estimators=500, max_depth=6, num_leaves=40, lr=0.05, subsample=0.8, colsample_bytree=0.8</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>24348</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>24951.72</v>
+      </c>
+      <c r="I5" s="8" t="n"/>
+      <c r="J5" s="8" t="n"/>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Worse than v3 XGBoost tuned. LightGBM not tuned yet — expected to improve with tuning.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>v4</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>v5</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>2026-04-21</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>LightGBM Default + Feature Eng</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Blend 45% XGB + 55% LightGBM Tuned</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>04_model_tuning.ipynb</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>Same 11 engineered features as v3. LightGBM with default params (no tuning).</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>n_estimators=500, max_depth=6, num_leaves=40, lr=0.05, subsample=0.8, colsample_bytree=0.8</t>
-        </is>
-      </c>
-      <c r="G6" s="8" t="n">
-        <v>24348</v>
-      </c>
-      <c r="H6" s="9" t="n">
-        <v>24951.72</v>
-      </c>
-      <c r="I6" s="8" t="n"/>
-      <c r="J6" s="8" t="n"/>
-      <c r="K6" s="8" t="inlineStr">
-        <is>
-          <t>Worse than v3 XGBoost tuned. LightGBM not tuned yet — expected to improve with tuning.</t>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Same 11 engineered features. Blend of tuned XGBoost + tuned LightGBM.</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>XGB: n_estimators=1000, max_depth=7, lr=0.05 | LGBM: n_estimators=1200, max_depth=8, num_leaves=80, lr=0.08</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>21570</v>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>22428.34</v>
+      </c>
+      <c r="I6" s="7" t="n"/>
+      <c r="J6" s="7" t="n"/>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>Best Kaggle score so far. Blending two models reduced variance. -1,372 vs v3.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>v5</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-21</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Blend 45% XGB + 55% LightGBM Tuned</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>04_model_tuning.ipynb</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>Same 11 engineered features. Blend of tuned XGBoost + tuned LightGBM.</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>XGB: n_estimators=1000, max_depth=7, lr=0.05 | LGBM: n_estimators=1200, max_depth=8, num_leaves=80, lr=0.08</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="n">
-        <v>21570</v>
-      </c>
-      <c r="H7" s="10" t="n">
-        <v>22428.34</v>
-      </c>
-      <c r="I7" s="7" t="n"/>
-      <c r="J7" s="7" t="n"/>
-      <c r="K7" s="7" t="inlineStr">
-        <is>
-          <t>Best Kaggle score so far. Blending two models reduced variance. -1,372 vs v3.</t>
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>v6</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>XGB+LGBM Blend (Log Target)</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>05_advanced_tuning.ipynb</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>+log1p target, OOF town_median_price, dist_x_storey, lease_x_area, log_dist_to_cbd</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>XGB: n_est=1000,depth=7,lr=0.05 | LGBM: tuned | blend ratio from search</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="n">
+        <v>21818</v>
+      </c>
+      <c r="H7" s="12" t="n">
+        <v>22124.05022</v>
+      </c>
+      <c r="I7" s="11" t="inlineStr"/>
+      <c r="J7" s="11" t="inlineStr"/>
+      <c r="K7" s="11" t="inlineStr">
+        <is>
+          <t>Log target + OOF encoding + interaction features. Best so far. -$304 vs v5.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: v7 model — stacking + street_freq (Kaggle RMSE 21,905)
- Add 06_stacking.ipynb: Ridge meta-model on OOF XGB+LGBM predictions,
  street_name frequency encoding, inline RandomizedSearchCV tuning
- Add sub_v7_stack.csv submission (Kaggle RMSE 21,905.74, OOF 21,841)
- Update submission tracker: add v7 as new best, downgrade v6
- Update README and CHANGELOG: v7 best, next steps updated
- CV-Kaggle gap collapsed from $306 (v6) to $64 (v7)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/submission_tracker.xlsx
+++ b/outputs/submission_tracker.xlsx
@@ -38,7 +38,7 @@
       <color rgb="00006100"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -68,6 +68,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -103,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -137,6 +149,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -502,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -801,47 +816,92 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>v6</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>2026-04-22</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t>XGB+LGBM Blend (Log Target)</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D7" s="13" t="inlineStr">
         <is>
           <t>05_advanced_tuning.ipynb</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E7" s="13" t="inlineStr">
         <is>
           <t>+log1p target, OOF town_median_price, dist_x_storey, lease_x_area, log_dist_to_cbd</t>
         </is>
       </c>
-      <c r="F7" s="11" t="inlineStr">
+      <c r="F7" s="13" t="inlineStr">
         <is>
           <t>XGB: n_est=1000,depth=7,lr=0.05 | LGBM: tuned | blend ratio from search</t>
         </is>
       </c>
-      <c r="G7" s="11" t="n">
+      <c r="G7" s="13" t="n">
         <v>21818</v>
       </c>
-      <c r="H7" s="12" t="n">
+      <c r="H7" s="14" t="n">
         <v>22124.05022</v>
       </c>
-      <c r="I7" s="11" t="inlineStr"/>
-      <c r="J7" s="11" t="inlineStr"/>
-      <c r="K7" s="11" t="inlineStr">
+      <c r="I7" s="13" t="inlineStr"/>
+      <c r="J7" s="13" t="inlineStr"/>
+      <c r="K7" s="13" t="inlineStr">
         <is>
           <t>Log target + OOF encoding + interaction features. Best so far. -$304 vs v5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>v7</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>Stacking + street_freq (XGB+LGBM OOF)</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>06_stacking.ipynb</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>+street_freq encoding, Ridge meta-model on OOF XGB+LGBM predictions</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>XGB: n_est=1500,depth=7,sub=0.9,col=0.6 | LGBM: n_est=1500,depth=10,leaves=80 | Ridge alpha=0.001</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="n">
+        <v>21841</v>
+      </c>
+      <c r="H8" s="15" t="n">
+        <v>21905.74292</v>
+      </c>
+      <c r="I8" s="15" t="n"/>
+      <c r="J8" s="15" t="n"/>
+      <c r="K8" s="15" t="inlineStr">
+        <is>
+          <t>Stacking + street_freq. New best. -$218 vs v6. CV-Kaggle gap collapsed $306→$64.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: v8 model — 3-model stack XGB+LGBM+ExtraTrees (Kaggle RMSE 21,805)
- Add ExtraTreesRegressor as 3rd base model in stacking pipeline
- Ridge meta-model on [xgb_oof, lgbm_oof, et_oof] — ET coef=0.22
- OOF RMSE improved $133 vs v7 ($21,708 vs $21,841)
- Kaggle RMSE: 21,804.67 — new best (-$101 vs v7)
- ET bagging diversity complements XGB/LGBM boosting models
- Add stacking_explained.html/.md self-study guides
- Update README, CHANGELOG, submission_tracker

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/submission_tracker.xlsx
+++ b/outputs/submission_tracker.xlsx
@@ -38,7 +38,7 @@
       <color rgb="00006100"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -82,6 +82,18 @@
         <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9C4"/>
+        <bgColor rgb="00FFF9C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C8E6C9"/>
+        <bgColor rgb="00C8E6C9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -115,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -152,6 +164,8 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -517,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -861,47 +875,92 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>v7</t>
         </is>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>2026-04-22</t>
         </is>
       </c>
-      <c r="C8" s="15" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
         <is>
           <t>Stacking + street_freq (XGB+LGBM OOF)</t>
         </is>
       </c>
-      <c r="D8" s="15" t="inlineStr">
+      <c r="D8" s="16" t="inlineStr">
         <is>
           <t>06_stacking.ipynb</t>
         </is>
       </c>
-      <c r="E8" s="15" t="inlineStr">
+      <c r="E8" s="16" t="inlineStr">
         <is>
           <t>+street_freq encoding, Ridge meta-model on OOF XGB+LGBM predictions</t>
         </is>
       </c>
-      <c r="F8" s="15" t="inlineStr">
+      <c r="F8" s="16" t="inlineStr">
         <is>
           <t>XGB: n_est=1500,depth=7,sub=0.9,col=0.6 | LGBM: n_est=1500,depth=10,leaves=80 | Ridge alpha=0.001</t>
         </is>
       </c>
-      <c r="G8" s="15" t="n">
+      <c r="G8" s="16" t="n">
         <v>21841</v>
       </c>
-      <c r="H8" s="15" t="n">
+      <c r="H8" s="16" t="n">
         <v>21905.74292</v>
       </c>
-      <c r="I8" s="15" t="n"/>
-      <c r="J8" s="15" t="n"/>
-      <c r="K8" s="15" t="inlineStr">
+      <c r="I8" s="16" t="n"/>
+      <c r="J8" s="16" t="n"/>
+      <c r="K8" s="16" t="inlineStr">
         <is>
           <t>Stacking + street_freq. New best. -$218 vs v6. CV-Kaggle gap collapsed $306→$64.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>v8</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>3-Model Stack (XGB + LGBM + Extra Trees OOF)</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>07_extra_trees_stack.ipynb</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>Same as v7 + ExtraTreesRegressor as 3rd base model</t>
+        </is>
+      </c>
+      <c r="F9" s="17" t="inlineStr">
+        <is>
+          <t>XGB: n_est=1500,depth=7,sub=0.9,col=0.6 | LGBM: n_est=1500,depth=10,leaves=80 | ET: n_est=700,max_feat=0.8 | Ridge alpha=0.001</t>
+        </is>
+      </c>
+      <c r="G9" s="17" t="n">
+        <v>21708</v>
+      </c>
+      <c r="H9" s="17" t="n">
+        <v>21804.66703</v>
+      </c>
+      <c r="I9" s="17" t="n"/>
+      <c r="J9" s="17" t="n"/>
+      <c r="K9" s="17" t="inlineStr">
+        <is>
+          <t>3-model stack. New best. -$101 vs v7. ET coef=0.22 (bagging diversity helped). Gap to 1st: $338.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: update Excel tracker and HTML journey through v17 and team ensemble
Add 14 new rows to submission_tracker.xlsx (v9–v17, team members, ensembles).
Update submission_journey.html: score card, timeline, all tables, 7 new version
cards, 9 new features, and updated What's Next section.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/submission_tracker.xlsx
+++ b/outputs/submission_tracker.xlsx
@@ -38,7 +38,7 @@
       <color rgb="00006100"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -94,8 +94,33 @@
         <bgColor rgb="00C8E6C9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEBEE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F5F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E3F2FD"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -123,11 +148,25 @@
         <color rgb="00BBBBBB"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00DDDDDD"/>
+      </left>
+      <right style="thin">
+        <color rgb="00DDDDDD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00DDDDDD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00DDDDDD"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -166,6 +205,36 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="12" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="13" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="14" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -531,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -961,6 +1030,612 @@
       <c r="K9" s="17" t="inlineStr">
         <is>
           <t>3-model stack. New best. -$101 vs v7. ET coef=0.22 (bagging diversity helped). Gap to 1st: $338.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>v9</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>4-Model Stack XGB+LGBM+ET (Expanded OOF)</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>08_v9_stack.ipynb</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>Added: postal_sector_median_price (OOF), flat_model_median_price (OOF)</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>XGB: n_est=1500,depth=7,sub=0.9,col=0.6 | LGBM: n_est=1500,depth=10,leaves=80 | ET: n_est=700,max_feat=0.8 | Ridge alpha=0.001</t>
+        </is>
+      </c>
+      <c r="G10" s="19" t="n">
+        <v>21708</v>
+      </c>
+      <c r="H10" s="19" t="n">
+        <v>21755.56</v>
+      </c>
+      <c r="I10" s="19" t="n"/>
+      <c r="J10" s="18" t="n"/>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>–$49 vs v8. Gap $47 (excellent). Postal sector OOF adds finer location signal than town.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>v10–v13</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>2026-04-23 to 04-27</t>
+        </is>
+      </c>
+      <c r="C11" s="20" t="inlineStr">
+        <is>
+          <t>HPO + H3/block/CatBoost experiments</t>
+        </is>
+      </c>
+      <c r="D11" s="20" t="inlineStr">
+        <is>
+          <t>09–13_*.ipynb</t>
+        </is>
+      </c>
+      <c r="E11" s="20" t="inlineStr">
+        <is>
+          <t>H3 geohash spatial encoding, block_num extraction, Optuna HPO, standalone CatBoost</t>
+        </is>
+      </c>
+      <c r="F11" s="20" t="inlineStr">
+        <is>
+          <t>Optuna Bayesian search (100 trials each XGB/LGBM); various CatBoost params</t>
+        </is>
+      </c>
+      <c r="G11" s="21" t="n">
+        <v>21578</v>
+      </c>
+      <c r="H11" s="21" t="n">
+        <v>21783.02</v>
+      </c>
+      <c r="I11" s="21" t="n"/>
+      <c r="J11" s="20" t="n"/>
+      <c r="K11" s="20" t="inlineStr">
+        <is>
+          <t>OOF improved vs v9 but Kaggle $21,783 worse. Test distribution drift or subtle leakage. Experiments informed v14b.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="22" t="inlineStr">
+        <is>
+          <t>v14b</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="C12" s="22" t="inlineStr">
+        <is>
+          <t>Lease Depreciation + Storey Interaction Features</t>
+        </is>
+      </c>
+      <c r="D12" s="22" t="inlineStr">
+        <is>
+          <t>14b_clean_features.ipynb</t>
+        </is>
+      </c>
+      <c r="E12" s="22" t="inlineStr">
+        <is>
+          <t>Added: log_remaining_lease, lease_below_60, lease_x_below60, flat_type_rank, storey_x_flattype</t>
+        </is>
+      </c>
+      <c r="F12" s="22" t="inlineStr">
+        <is>
+          <t>Same as v9 base model params</t>
+        </is>
+      </c>
+      <c r="G12" s="23" t="n">
+        <v>21593</v>
+      </c>
+      <c r="H12" s="23" t="n"/>
+      <c r="I12" s="23" t="n"/>
+      <c r="J12" s="22" t="n"/>
+      <c r="K12" s="22" t="inlineStr">
+        <is>
+          <t>5 new interaction features. Not individually submitted to Kaggle — folded into v15.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="22" t="inlineStr">
+        <is>
+          <t>v15</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="C13" s="22" t="inlineStr">
+        <is>
+          <t>town×flat_type + Transaction Year OOF Encodings</t>
+        </is>
+      </c>
+      <c r="D13" s="22" t="inlineStr">
+        <is>
+          <t>15_interaction_oofs.ipynb</t>
+        </is>
+      </c>
+      <c r="E13" s="22" t="inlineStr">
+        <is>
+          <t>Added: town_flat_type_median_price (OOF), year_median_price (OOF); built on v14b features</t>
+        </is>
+      </c>
+      <c r="F13" s="22" t="inlineStr">
+        <is>
+          <t>5 ENCODE_PAIRS total; Ridge alpha=0.001</t>
+        </is>
+      </c>
+      <c r="G13" s="23" t="n">
+        <v>21593</v>
+      </c>
+      <c r="H13" s="23" t="n"/>
+      <c r="I13" s="23" t="n"/>
+      <c r="J13" s="22" t="n"/>
+      <c r="K13" s="22" t="inlineStr">
+        <is>
+          <t>–$115 OOF vs v9. Team submission only (20260428_21593_MengHai.csv). No individual Kaggle score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="24" t="inlineStr">
+        <is>
+          <t>v16</t>
+        </is>
+      </c>
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="C14" s="24" t="inlineStr">
+        <is>
+          <t>4-Model Stack: CatBoost as 4th Base + 100% Retrain</t>
+        </is>
+      </c>
+      <c r="D14" s="24" t="inlineStr">
+        <is>
+          <t>16_catboost_stack.ipynb</t>
+        </is>
+      </c>
+      <c r="E14" s="24" t="inlineStr">
+        <is>
+          <t>Added: CatBoostRegressor (4th base, symmetric trees); 100% data retrain file also generated</t>
+        </is>
+      </c>
+      <c r="F14" s="24" t="inlineStr">
+        <is>
+          <t>CAT: iterations=1000,depth=7,lr=0.08,l2=1,col=0.7 | Ridge alpha=0.001 | XGB 0.343, LGBM 0.367, ET 0.120, CAT 0.173</t>
+        </is>
+      </c>
+      <c r="G14" s="25" t="n">
+        <v>21552</v>
+      </c>
+      <c r="H14" s="25" t="n"/>
+      <c r="I14" s="25" t="n"/>
+      <c r="J14" s="24" t="n"/>
+      <c r="K14" s="24" t="inlineStr">
+        <is>
+          <t>Best solo OOF $21,552. CatBoost structural diversity (symmetric trees) added real value. Used as MengHai contribution to team ensemble.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>v17</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="C15" s="20" t="inlineStr">
+        <is>
+          <t>School Name OOF Encoding (Rejected)</t>
+        </is>
+      </c>
+      <c r="D15" s="20" t="inlineStr">
+        <is>
+          <t>17_school_oof.ipynb</t>
+        </is>
+      </c>
+      <c r="E15" s="20" t="inlineStr">
+        <is>
+          <t>Added: pri_sch_median_price (OOF, 177 schools), log_pri_sch_dist, log_sec_sch_dist</t>
+        </is>
+      </c>
+      <c r="F15" s="20" t="inlineStr">
+        <is>
+          <t>6 ENCODE_PAIRS; same base params as v16</t>
+        </is>
+      </c>
+      <c r="G15" s="21" t="n">
+        <v>21556</v>
+      </c>
+      <c r="H15" s="21" t="n"/>
+      <c r="I15" s="21" t="n"/>
+      <c r="J15" s="20" t="n"/>
+      <c r="K15" s="20" t="inlineStr">
+        <is>
+          <t>OOF $21,556 — $4 worse than v16. School signal already captured by postal_sector_median_price (598 groups). Rejected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="22" t="inlineStr">
+        <is>
+          <t>Likhong-v1</t>
+        </is>
+      </c>
+      <c r="B16" s="22" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="C16" s="22" t="inlineStr">
+        <is>
+          <t>Unknown model (team member)</t>
+        </is>
+      </c>
+      <c r="D16" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E16" s="22" t="inlineStr">
+        <is>
+          <t>Details not available</t>
+        </is>
+      </c>
+      <c r="F16" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" s="23" t="n"/>
+      <c r="H16" s="23" t="n">
+        <v>22187.95</v>
+      </c>
+      <c r="I16" s="23" t="n"/>
+      <c r="J16" s="22" t="n"/>
+      <c r="K16" s="22" t="inlineStr">
+        <is>
+          <t>Team member submission. Model details not available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="22" t="inlineStr">
+        <is>
+          <t>Lanson-v1</t>
+        </is>
+      </c>
+      <c r="B17" s="22" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="C17" s="22" t="inlineStr">
+        <is>
+          <t>Unknown model (team member)</t>
+        </is>
+      </c>
+      <c r="D17" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E17" s="22" t="inlineStr">
+        <is>
+          <t>Details not available</t>
+        </is>
+      </c>
+      <c r="F17" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G17" s="23" t="n"/>
+      <c r="H17" s="23" t="n">
+        <v>21932.24</v>
+      </c>
+      <c r="I17" s="23" t="n"/>
+      <c r="J17" s="22" t="n"/>
+      <c r="K17" s="22" t="inlineStr">
+        <is>
+          <t>Team member submission. Model details not available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="22" t="inlineStr">
+        <is>
+          <t>Lanson-v2</t>
+        </is>
+      </c>
+      <c r="B18" s="22" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="C18" s="22" t="inlineStr">
+        <is>
+          <t>Unknown model (team member)</t>
+        </is>
+      </c>
+      <c r="D18" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E18" s="22" t="inlineStr">
+        <is>
+          <t>Details not available</t>
+        </is>
+      </c>
+      <c r="F18" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G18" s="23" t="n"/>
+      <c r="H18" s="23" t="n">
+        <v>21705.81</v>
+      </c>
+      <c r="I18" s="23" t="n"/>
+      <c r="J18" s="22" t="n"/>
+      <c r="K18" s="22" t="inlineStr">
+        <is>
+          <t>Team member submission. Details not available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>Lai-v1</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="C19" s="20" t="inlineStr">
+        <is>
+          <t>Unknown model (team member — malformed)</t>
+        </is>
+      </c>
+      <c r="D19" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E19" s="20" t="inlineStr">
+        <is>
+          <t>Details not available</t>
+        </is>
+      </c>
+      <c r="F19" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G19" s="21" t="n"/>
+      <c r="H19" s="21" t="n">
+        <v>35111.47</v>
+      </c>
+      <c r="I19" s="21" t="n"/>
+      <c r="J19" s="20" t="n"/>
+      <c r="K19" s="20" t="inlineStr">
+        <is>
+          <t>Team member. Malformed submission format — score not meaningful.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="22" t="inlineStr">
+        <is>
+          <t>Lanson-full</t>
+        </is>
+      </c>
+      <c r="B20" s="22" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="C20" s="22" t="inlineStr">
+        <is>
+          <t>Unknown — likely 100% data retrain (team member)</t>
+        </is>
+      </c>
+      <c r="D20" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E20" s="22" t="inlineStr">
+        <is>
+          <t>Details not available</t>
+        </is>
+      </c>
+      <c r="F20" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G20" s="23" t="n"/>
+      <c r="H20" s="23" t="n">
+        <v>21548.25</v>
+      </c>
+      <c r="I20" s="23" t="n"/>
+      <c r="J20" s="22" t="n"/>
+      <c r="K20" s="22" t="inlineStr">
+        <is>
+          <t>Team member (Lanson). Best individual team submission before ensemble.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>Ensemble-eq</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="C21" s="26" t="inlineStr">
+        <is>
+          <t>Equal-weight 3-model team blend</t>
+        </is>
+      </c>
+      <c r="D21" s="26" t="inlineStr">
+        <is>
+          <t>ensemble_team.ipynb</t>
+        </is>
+      </c>
+      <c r="E21" s="26" t="inlineStr">
+        <is>
+          <t>Equal-weight average of MengHai (v16), Lanson (full), Likhong predictions</t>
+        </is>
+      </c>
+      <c r="F21" s="26" t="inlineStr">
+        <is>
+          <t>Equal weights (1/3 each)</t>
+        </is>
+      </c>
+      <c r="G21" s="27" t="n"/>
+      <c r="H21" s="27" t="n">
+        <v>21359.82</v>
+      </c>
+      <c r="I21" s="27" t="n"/>
+      <c r="J21" s="26" t="n"/>
+      <c r="K21" s="26" t="inlineStr">
+        <is>
+          <t>–$188 vs best individual. Error cancellation across diverse models.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="24" t="inlineStr">
+        <is>
+          <t>Ensemble-wt</t>
+        </is>
+      </c>
+      <c r="B22" s="24" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="C22" s="24" t="inlineStr">
+        <is>
+          <t>Weighted 3-model team blend (Ridge-optimised) — BEST</t>
+        </is>
+      </c>
+      <c r="D22" s="24" t="inlineStr">
+        <is>
+          <t>ensemble_team.ipynb</t>
+        </is>
+      </c>
+      <c r="E22" s="24" t="inlineStr">
+        <is>
+          <t>Weighted average of MengHai (v16), Lanson (full), Likhong — weights via Ridge on OOF</t>
+        </is>
+      </c>
+      <c r="F22" s="24" t="inlineStr">
+        <is>
+          <t>Ridge meta on OOF predictions; optimised weights</t>
+        </is>
+      </c>
+      <c r="G22" s="25" t="n"/>
+      <c r="H22" s="25" t="n">
+        <v>21350.91</v>
+      </c>
+      <c r="I22" s="25" t="n"/>
+      <c r="J22" s="24" t="n"/>
+      <c r="K22" s="24" t="inlineStr">
+        <is>
+          <t>BEST! #2 on Kaggle leaderboard. Gap to 1st (Group 9): $108. –$197 vs best individual submission.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="26" t="inlineStr">
+        <is>
+          <t>Ensemble-rk</t>
+        </is>
+      </c>
+      <c r="B23" s="26" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="C23" s="26" t="inlineStr">
+        <is>
+          <t>Rank-average 3-model team blend</t>
+        </is>
+      </c>
+      <c r="D23" s="26" t="inlineStr">
+        <is>
+          <t>ensemble_team.ipynb</t>
+        </is>
+      </c>
+      <c r="E23" s="26" t="inlineStr">
+        <is>
+          <t>Rank-average of MengHai (v16), Lanson (full), Likhong predictions</t>
+        </is>
+      </c>
+      <c r="F23" s="26" t="inlineStr">
+        <is>
+          <t>Rank averaging (convert to ranks, then average)</t>
+        </is>
+      </c>
+      <c r="G23" s="27" t="n"/>
+      <c r="H23" s="27" t="n">
+        <v>21384.22</v>
+      </c>
+      <c r="I23" s="27" t="n"/>
+      <c r="J23" s="26" t="n"/>
+      <c r="K23" s="26" t="inlineStr">
+        <is>
+          <t>–$164 vs best individual.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: change Lai-v1 status from malformed to team across all trackers
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/submission_tracker.xlsx
+++ b/outputs/submission_tracker.xlsx
@@ -1425,45 +1425,45 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="20" t="inlineStr">
+      <c r="A19" s="22" t="inlineStr">
         <is>
           <t>Lai-v1</t>
         </is>
       </c>
-      <c r="B19" s="20" t="inlineStr">
+      <c r="B19" s="22" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="C19" s="20" t="inlineStr">
+      <c r="C19" s="22" t="inlineStr">
         <is>
           <t>Unknown model (team member — malformed)</t>
         </is>
       </c>
-      <c r="D19" s="20" t="inlineStr">
+      <c r="D19" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E19" s="20" t="inlineStr">
+      <c r="E19" s="22" t="inlineStr">
         <is>
           <t>Details not available</t>
         </is>
       </c>
-      <c r="F19" s="20" t="inlineStr">
+      <c r="F19" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G19" s="21" t="n"/>
-      <c r="H19" s="21" t="n">
+      <c r="G19" s="23" t="n"/>
+      <c r="H19" s="23" t="n">
         <v>35111.47</v>
       </c>
-      <c r="I19" s="21" t="n"/>
-      <c r="J19" s="20" t="n"/>
-      <c r="K19" s="20" t="inlineStr">
-        <is>
-          <t>Team member. Malformed submission format — score not meaningful.</t>
+      <c r="I19" s="23" t="n"/>
+      <c r="J19" s="22" t="n"/>
+      <c r="K19" s="22" t="inlineStr">
+        <is>
+          <t>Team member submission. Details not available.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: add Likhong-v0a/v0b entries to match Kaggle's 21 submissions
Two early Likhong submission.csv entries (both $23,299.17, Apr 21) were
missing from all 3 trackers. Submission count updated 19 → 21.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/submission_tracker.xlsx
+++ b/outputs/submission_tracker.xlsx
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1298,93 +1298,93 @@
     <row r="16">
       <c r="A16" s="22" t="inlineStr">
         <is>
-          <t>Likhong-v1</t>
+          <t>Likhong-v0a</t>
         </is>
       </c>
       <c r="B16" s="22" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="C16" s="22" t="inlineStr">
         <is>
-          <t>Unknown model (team member)</t>
+          <t>Unknown model — 1st attempt (team member)</t>
         </is>
       </c>
       <c r="D16" s="22" t="inlineStr">
         <is>
+          <t>submission.csv</t>
+        </is>
+      </c>
+      <c r="E16" s="22" t="inlineStr">
+        <is>
+          <t>Details not available</t>
+        </is>
+      </c>
+      <c r="F16" s="22" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E16" s="22" t="inlineStr">
-        <is>
-          <t>Details not available</t>
-        </is>
-      </c>
-      <c r="F16" s="22" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G16" s="23" t="n"/>
+      <c r="G16" s="22" t="n"/>
       <c r="H16" s="23" t="n">
-        <v>22187.95</v>
-      </c>
-      <c r="I16" s="23" t="n"/>
+        <v>23299.17</v>
+      </c>
+      <c r="I16" s="22" t="n"/>
       <c r="J16" s="22" t="n"/>
       <c r="K16" s="22" t="inlineStr">
         <is>
-          <t>Team member submission. Model details not available.</t>
+          <t>Eng Lik Hong's first Kaggle submission. Details not available. File: submission.csv (try only).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="22" t="inlineStr">
         <is>
-          <t>Lanson-v1</t>
+          <t>Likhong-v0b</t>
         </is>
       </c>
       <c r="B17" s="22" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="C17" s="22" t="inlineStr">
         <is>
-          <t>Unknown model (team member)</t>
+          <t>Unknown model — 2nd attempt (team member)</t>
         </is>
       </c>
       <c r="D17" s="22" t="inlineStr">
         <is>
+          <t>submission.csv</t>
+        </is>
+      </c>
+      <c r="E17" s="22" t="inlineStr">
+        <is>
+          <t>Details not available</t>
+        </is>
+      </c>
+      <c r="F17" s="22" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E17" s="22" t="inlineStr">
-        <is>
-          <t>Details not available</t>
-        </is>
-      </c>
-      <c r="F17" s="22" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G17" s="23" t="n"/>
+      <c r="G17" s="22" t="n"/>
       <c r="H17" s="23" t="n">
-        <v>21932.24</v>
-      </c>
-      <c r="I17" s="23" t="n"/>
+        <v>23299.17</v>
+      </c>
+      <c r="I17" s="22" t="n"/>
       <c r="J17" s="22" t="n"/>
       <c r="K17" s="22" t="inlineStr">
         <is>
-          <t>Team member submission. Model details not available.</t>
+          <t>Eng Lik Hong's second Kaggle submission. Same score as v0a. File: submission.csv (try2).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="22" t="inlineStr">
         <is>
-          <t>Lanson-v2</t>
+          <t>Likhong-v1</t>
         </is>
       </c>
       <c r="B18" s="22" t="inlineStr">
@@ -1414,30 +1414,30 @@
       </c>
       <c r="G18" s="23" t="n"/>
       <c r="H18" s="23" t="n">
-        <v>21705.81</v>
+        <v>22187.95</v>
       </c>
       <c r="I18" s="23" t="n"/>
       <c r="J18" s="22" t="n"/>
       <c r="K18" s="22" t="inlineStr">
         <is>
-          <t>Team member submission. Details not available.</t>
+          <t>Team member submission. Model details not available.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="22" t="inlineStr">
         <is>
-          <t>Lai-v1</t>
+          <t>Lanson-v1</t>
         </is>
       </c>
       <c r="B19" s="22" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="C19" s="22" t="inlineStr">
         <is>
-          <t>Unknown model (team member — malformed)</t>
+          <t>Unknown model (team member)</t>
         </is>
       </c>
       <c r="D19" s="22" t="inlineStr">
@@ -1457,30 +1457,30 @@
       </c>
       <c r="G19" s="23" t="n"/>
       <c r="H19" s="23" t="n">
-        <v>35111.47</v>
+        <v>21932.24</v>
       </c>
       <c r="I19" s="23" t="n"/>
       <c r="J19" s="22" t="n"/>
       <c r="K19" s="22" t="inlineStr">
         <is>
-          <t>Team member submission. Details not available.</t>
+          <t>Team member submission. Model details not available.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="22" t="inlineStr">
         <is>
-          <t>Lanson-full</t>
+          <t>Lanson-v2</t>
         </is>
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="C20" s="22" t="inlineStr">
         <is>
-          <t>Unknown — likely 100% data retrain (team member)</t>
+          <t>Unknown model (team member)</t>
         </is>
       </c>
       <c r="D20" s="22" t="inlineStr">
@@ -1500,106 +1500,106 @@
       </c>
       <c r="G20" s="23" t="n"/>
       <c r="H20" s="23" t="n">
-        <v>21548.25</v>
+        <v>21705.81</v>
       </c>
       <c r="I20" s="23" t="n"/>
       <c r="J20" s="22" t="n"/>
       <c r="K20" s="22" t="inlineStr">
         <is>
+          <t>Team member submission. Details not available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="22" t="inlineStr">
+        <is>
+          <t>Lai-v1</t>
+        </is>
+      </c>
+      <c r="B21" s="22" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="C21" s="22" t="inlineStr">
+        <is>
+          <t>Unknown model (team member — malformed)</t>
+        </is>
+      </c>
+      <c r="D21" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" s="22" t="inlineStr">
+        <is>
+          <t>Details not available</t>
+        </is>
+      </c>
+      <c r="F21" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" s="23" t="n"/>
+      <c r="H21" s="23" t="n">
+        <v>35111.47</v>
+      </c>
+      <c r="I21" s="23" t="n"/>
+      <c r="J21" s="22" t="n"/>
+      <c r="K21" s="22" t="inlineStr">
+        <is>
+          <t>Team member submission. Details not available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="22" t="inlineStr">
+        <is>
+          <t>Lanson-full</t>
+        </is>
+      </c>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="C22" s="22" t="inlineStr">
+        <is>
+          <t>Unknown — likely 100% data retrain (team member)</t>
+        </is>
+      </c>
+      <c r="D22" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E22" s="22" t="inlineStr">
+        <is>
+          <t>Details not available</t>
+        </is>
+      </c>
+      <c r="F22" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G22" s="23" t="n"/>
+      <c r="H22" s="23" t="n">
+        <v>21548.25</v>
+      </c>
+      <c r="I22" s="23" t="n"/>
+      <c r="J22" s="22" t="n"/>
+      <c r="K22" s="22" t="inlineStr">
+        <is>
           <t>Team member (Lanson). Best individual team submission before ensemble.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="26" t="inlineStr">
-        <is>
-          <t>Ensemble-eq</t>
-        </is>
-      </c>
-      <c r="B21" s="26" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-      <c r="C21" s="26" t="inlineStr">
-        <is>
-          <t>Equal-weight 3-model team blend</t>
-        </is>
-      </c>
-      <c r="D21" s="26" t="inlineStr">
-        <is>
-          <t>ensemble_team.ipynb</t>
-        </is>
-      </c>
-      <c r="E21" s="26" t="inlineStr">
-        <is>
-          <t>Equal-weight average of MengHai (v16), Lanson (full), Likhong predictions</t>
-        </is>
-      </c>
-      <c r="F21" s="26" t="inlineStr">
-        <is>
-          <t>Equal weights (1/3 each)</t>
-        </is>
-      </c>
-      <c r="G21" s="27" t="n"/>
-      <c r="H21" s="27" t="n">
-        <v>21359.82</v>
-      </c>
-      <c r="I21" s="27" t="n"/>
-      <c r="J21" s="26" t="n"/>
-      <c r="K21" s="26" t="inlineStr">
-        <is>
-          <t>–$188 vs best individual. Error cancellation across diverse models.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="24" t="inlineStr">
-        <is>
-          <t>Ensemble-wt</t>
-        </is>
-      </c>
-      <c r="B22" s="24" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-      <c r="C22" s="24" t="inlineStr">
-        <is>
-          <t>Weighted 3-model team blend (Ridge-optimised) — BEST</t>
-        </is>
-      </c>
-      <c r="D22" s="24" t="inlineStr">
-        <is>
-          <t>ensemble_team.ipynb</t>
-        </is>
-      </c>
-      <c r="E22" s="24" t="inlineStr">
-        <is>
-          <t>Weighted average of MengHai (v16), Lanson (full), Likhong — weights via Ridge on OOF</t>
-        </is>
-      </c>
-      <c r="F22" s="24" t="inlineStr">
-        <is>
-          <t>Ridge meta on OOF predictions; optimised weights</t>
-        </is>
-      </c>
-      <c r="G22" s="25" t="n"/>
-      <c r="H22" s="25" t="n">
-        <v>21350.91</v>
-      </c>
-      <c r="I22" s="25" t="n"/>
-      <c r="J22" s="24" t="n"/>
-      <c r="K22" s="24" t="inlineStr">
-        <is>
-          <t>BEST! #2 on Kaggle leaderboard. Gap to 1st (Group 9): $108. –$197 vs best individual submission.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t>Ensemble-rk</t>
+          <t>Ensemble-eq</t>
         </is>
       </c>
       <c r="B23" s="26" t="inlineStr">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="C23" s="26" t="inlineStr">
         <is>
-          <t>Rank-average 3-model team blend</t>
+          <t>Equal-weight 3-model team blend</t>
         </is>
       </c>
       <c r="D23" s="26" t="inlineStr">
@@ -1619,21 +1619,107 @@
       </c>
       <c r="E23" s="26" t="inlineStr">
         <is>
-          <t>Rank-average of MengHai (v16), Lanson (full), Likhong predictions</t>
+          <t>Equal-weight average of MengHai (v16), Lanson (full), Likhong predictions</t>
         </is>
       </c>
       <c r="F23" s="26" t="inlineStr">
         <is>
-          <t>Rank averaging (convert to ranks, then average)</t>
+          <t>Equal weights (1/3 each)</t>
         </is>
       </c>
       <c r="G23" s="27" t="n"/>
       <c r="H23" s="27" t="n">
-        <v>21384.22</v>
+        <v>21359.82</v>
       </c>
       <c r="I23" s="27" t="n"/>
       <c r="J23" s="26" t="n"/>
       <c r="K23" s="26" t="inlineStr">
+        <is>
+          <t>–$188 vs best individual. Error cancellation across diverse models.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="24" t="inlineStr">
+        <is>
+          <t>Ensemble-wt</t>
+        </is>
+      </c>
+      <c r="B24" s="24" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="C24" s="24" t="inlineStr">
+        <is>
+          <t>Weighted 3-model team blend (Ridge-optimised) — BEST</t>
+        </is>
+      </c>
+      <c r="D24" s="24" t="inlineStr">
+        <is>
+          <t>ensemble_team.ipynb</t>
+        </is>
+      </c>
+      <c r="E24" s="24" t="inlineStr">
+        <is>
+          <t>Weighted average of MengHai (v16), Lanson (full), Likhong — weights via Ridge on OOF</t>
+        </is>
+      </c>
+      <c r="F24" s="24" t="inlineStr">
+        <is>
+          <t>Ridge meta on OOF predictions; optimised weights</t>
+        </is>
+      </c>
+      <c r="G24" s="25" t="n"/>
+      <c r="H24" s="25" t="n">
+        <v>21350.91</v>
+      </c>
+      <c r="I24" s="25" t="n"/>
+      <c r="J24" s="24" t="n"/>
+      <c r="K24" s="24" t="inlineStr">
+        <is>
+          <t>BEST! #2 on Kaggle leaderboard. Gap to 1st (Group 9): $108. –$197 vs best individual submission.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="26" t="inlineStr">
+        <is>
+          <t>Ensemble-rk</t>
+        </is>
+      </c>
+      <c r="B25" s="26" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="C25" s="26" t="inlineStr">
+        <is>
+          <t>Rank-average 3-model team blend</t>
+        </is>
+      </c>
+      <c r="D25" s="26" t="inlineStr">
+        <is>
+          <t>ensemble_team.ipynb</t>
+        </is>
+      </c>
+      <c r="E25" s="26" t="inlineStr">
+        <is>
+          <t>Rank-average of MengHai (v16), Lanson (full), Likhong predictions</t>
+        </is>
+      </c>
+      <c r="F25" s="26" t="inlineStr">
+        <is>
+          <t>Rank averaging (convert to ranks, then average)</t>
+        </is>
+      </c>
+      <c r="G25" s="27" t="n"/>
+      <c r="H25" s="27" t="n">
+        <v>21384.22</v>
+      </c>
+      <c r="I25" s="27" t="n"/>
+      <c r="J25" s="26" t="n"/>
+      <c r="K25" s="26" t="inlineStr">
         <is>
           <t>–$164 vs best individual.</t>
         </is>

</xml_diff>

<commit_message>
feat: v19/v20 Optuna experiments, Ken Lai ensemble, new best $21,335.57
Experiments:
- nb19: LGBM+ET Optuna params → stack OOF $21,533 (–$19 vs v16)
- nb20: CatBoost Optuna 100-trial TPE → individual val $21,484 (–$1,123)
- nb21/v20: all Optuna params → OOF $21,465 but Kaggle $21,827 (overfit, gap $362)

Team ensemble (ensemble_team.ipynb):
- Ens-2: 4-member with Ken Lai — rank avg generated, weighted $21,660.70 (Lai scale drag)
- Ens-3: 3-member v20 — equal $21,345.60, weighted $21,335.57 NEW BEST (gap to 1st ~$93)

Tracker updates:
- submission_tracker.xlsx: all Apr 29 results logged
- submission_journey.html: full timeline, QR table, version cards (v19, v20, Ens-1–3), What's Next
- webapp/index.html: best RMSE $21,335.57, gap ~$93, improvement –$4,607
- webapp/search_index.json: all snippets refreshed
- webapp/pipeline_automation_explained.html: new study guide

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/submission_tracker.xlsx
+++ b/outputs/submission_tracker.xlsx
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1722,6 +1722,209 @@
       <c r="K25" s="26" t="inlineStr">
         <is>
           <t>–$164 vs best individual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>3member-v19</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Equal-weight 3-model team blend (MengHai v19 upgrade)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>ensemble_team.ipynb</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Equal-weight average of MengHai (v19 Optuna LGBM+ET, OOF $21,533), Lanson (full), Likhong</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Equal weights (1/3 each)</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>21366.39</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>MengHai upgraded to v19 (Optuna LGBM+ET params). –$181 vs best individual. Slightly worse than yesterday 3-member-wt ($21,350.91).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>4member-wt</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Weighted 4-model team blend (incl. Ken Lai, 1/RMSE²) — FAILED</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>ensemble_team.ipynb</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Weighted average of MengHai (v19), Lanson (full), Likhong, Ken Lai — weights by 1/RMSE²</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Lai weight ~11% (1/35328²), others ~28–31% each</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>21660.7</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>WORSE. Lai's absolute predictions are ~$14K above market. At 11% weight, adds ~$1,500 upward bias to every prediction. Raw averaging cannot neutralise absolute scale errors — use rank averaging instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>v20</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>4-model stack — All Optuna params (XGB + LGBM Optuna + ET Optuna + CatBoost Optuna)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>21_all_optuna_params.ipynb</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Same 78 features as v19. All 4 base models with Optuna-tuned hyperparameters.</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>XGB: unchanged. LGBM: n_est=888, lr=0.0272, num_leaves=317. ET: n_est=600, depth=24. CatBoost: iterations=1994, depth=10, lr=0.0585.</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>21465</v>
+      </c>
+      <c r="H28" t="n">
+        <v>21826.58</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>OOF $21,465 but Kaggle $21,827 — gap $362 (unusually large). CatBoost Optuna params (depth=10, 1994 iter) tuned on 80/20 split likely overfit; Ridge over-weighted CatBoost at 36.6% amplified the issue. Worse than current best ($21,350.91). Do not use v20 individually; test in team ensemble to see if diversity still helps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>3member-equal-v20</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Equal-weight 3-model team blend (MengHai v20)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>ensemble_team.ipynb</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Equal-weight average of MengHai (v20, Kaggle $21,827), Lanson (full, $21,035), Likhong ($22,094)</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Equal weights (1/3 each). Lai excluded.</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
+        <v>21345.6</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>NEW BEST! $21,345.60 — beats previous best $21,350.91 by $5.31. Gap to 1st (Group 9 $21,242.91): ~$103. Equal-weight beat weighted — v20 errors partially uncorrelated with Lanson/Likhong despite worse individual score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>3member-wt-v20</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Weighted 3-model team blend (MengHai v20, 1/RMSE²)</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>ensemble_team.ipynb</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Weighted average of MengHai v20 ($21,827), Lanson ($21,035), Likhong ($22,094). Lai excluded.</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>1/RMSE² weights: Lanson ~36%, MengHai ~34%, Likhong ~30%.</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>21335.57</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>NEW BEST! $21,335.57 — beats prev best $21,345.60 by $10.03. Gap to 1st (Group 9 $21,242.91): ~$93. Weighted blend edged out equal-weight by $10 — Lanson higher weight paid off.</t>
         </is>
       </c>
     </row>

</xml_diff>